<commit_message>
Feat: added mandatory skin care details form, GitHub CI/CD Auto-Deploy, and update notification banner system
</commit_message>
<xml_diff>
--- a/DermaSense_Web_Test_Report.xlsx
+++ b/DermaSense_Web_Test_Report.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,18 +57,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B71C1C"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00E65100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
@@ -79,7 +67,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -120,18 +108,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FAFAFA"/>
         <bgColor rgb="00FAFAFA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEBEE"/>
-        <bgColor rgb="00FFEBEE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3E0"/>
-        <bgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -185,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -211,49 +187,43 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -646,7 +616,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-11  14:42:52   |   URL: https://dermasense-ai-18698.web.app   |   Total: 20   |   PASS: 10   FAIL: 2   SKIP: 8   NOT RUN: 0   Pass Rate: 50.0%</t>
+          <t>Generated: 2026-06-14  15:03:39   |   URL: https://dermasense-ai-18698.web.app   |   Total: 20   |   PASS: 20   FAIL: 0   SKIP: 0   NOT RUN: 0   Pass Rate: 100.0%</t>
         </is>
       </c>
     </row>
@@ -735,12 +705,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>5.96</t>
+          <t>8.27</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>14:24:35</t>
+          <t>14:58:21</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -787,12 +757,12 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>5.41</t>
+          <t>5.37</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>14:24:41</t>
+          <t>14:58:29</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
@@ -822,14 +792,14 @@
           <t>Login page has email field or sign-in elements</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>[FAIL]</t>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Login page elements not found</t>
+          <t>Login page detected — sign-in elements present</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -839,12 +809,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>36.48</t>
+          <t>31.69</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>14:24:46</t>
+          <t>14:58:35</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -874,14 +844,14 @@
           <t>Email input field is accessible and accepts text</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Email field not interactable (Flutter canvas may block direct input)</t>
+          <t>Email field accepts input</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -891,12 +861,12 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>102.94</t>
+          <t>32.32</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>14:25:23</t>
+          <t>14:59:07</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
@@ -926,14 +896,14 @@
           <t>Password field is accessible and accepts text (masked)</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Password field not directly interactable</t>
+          <t>Password field accepts input</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -943,12 +913,12 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>87.08</t>
+          <t>6.91</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>14:27:06</t>
+          <t>14:59:39</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -978,32 +948,29 @@
           <t>Wrong credentials display error message, stay on login</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>[FAIL]</t>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> "C:\Users\Praveenkumar S\Documents\pdd\kingrat\derma_sense_ai\selenium_tests\run_web_tests.py", line 341, in tc006
-    raise AssertionError("App redirected away with invalid credentials")
-AssertionError: App redirected away with invalid credentials
-</t>
+          <t>Stayed on login page (correct behavior, no redirect)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>App redirected away with invalid credentials</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>315.02</t>
+          <t>46.31</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>14:28:33</t>
+          <t>14:59:46</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
@@ -1013,7 +980,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>C:\Users\Praveenkumar S\Documents\pdd\kingrat\derma_sense_ai\selenium_tests\screenshots\143348_TC006.png</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1007,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>No explicit validation UI (acceptable for Flutter web)</t>
+          <t>Validation shown or stayed on login for empty email</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1050,12 +1017,12 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>311.54</t>
+          <t>43.72</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>14:33:48</t>
+          <t>15:00:32</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1085,14 +1052,14 @@
           <t>Forgot Password link exists on login page</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Forgot Password link not found (may need scroll or flutter semantics)</t>
+          <t>Forgot Password link found</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -1102,12 +1069,12 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>27.54</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>14:38:59</t>
+          <t>15:01:16</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
@@ -1137,14 +1104,14 @@
           <t>Sign Up link is present and clickable</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Sign Up link not found on page</t>
+          <t>Sign Up navigated to register. URL changed: True</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1154,12 +1121,12 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>27.42</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>14:39:27</t>
+          <t>15:01:22</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -1189,14 +1156,14 @@
           <t>Guest Access / Instant Access button visible</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Guest Access button not found</t>
+          <t>Guest Access button found</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -1206,12 +1173,12 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>48.64</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>14:39:54</t>
+          <t>15:01:34</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -1241,14 +1208,14 @@
           <t>Guest login button bypasses auth and opens dashboard</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Guest button not found/clickable</t>
+          <t>Dashboard loaded after Guest login. URL=https://dermasense-ai-18698.web.app/#/dashboard</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1258,17 +1225,17 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>48.64</t>
+          <t>11.93</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>14:40:43</t>
+          <t>15:01:40</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>https://dermasense-ai-18698.web.app/#/login</t>
+          <t>https://dermasense-ai-18698.web.app/#/dashboard</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1293,14 +1260,14 @@
           <t>Valid email + password login reaches Dashboard</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>No credentials provided — re-run with --email and --password</t>
+          <t>Login successful with test@dermasense.ai. URL=https://dermasense-ai-18698.web.app/#/dashboard</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1310,17 +1277,17 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>40.23</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>14:41:32</t>
+          <t>15:01:52</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>https://dermasense-ai-18698.web.app/#/login</t>
+          <t>https://dermasense-ai-18698.web.app/#/dashboard</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -1352,7 +1319,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Mobile responsive — scrollWidth=482, viewportWidth=482</t>
+          <t>Mobile responsive — scrollWidth=500, viewportWidth=500</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1362,12 +1329,12 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>7.79</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>14:41:32</t>
+          <t>15:02:33</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1404,7 +1371,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>HTTPS confirmed: https://dermasense-ai-18698.web.app/#/login</t>
+          <t>HTTPS confirmed: https://dermasense-ai-18698.web.app/</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -1414,12 +1381,12 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>4.25</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>14:41:40</t>
+          <t>15:02:41</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
@@ -1456,7 +1423,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Page loaded in 3.32s</t>
+          <t>Page loaded in 3.5s</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1466,12 +1433,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>3.32</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>14:41:44</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1501,14 +1468,14 @@
           <t>Google Sign-In button visible on login page</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>[SKIP]</t>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>[PASS]</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Google button not found (may not be visible on web build)</t>
+          <t>Google Sign-In button found</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1518,12 +1485,12 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>38.01</t>
+          <t>7.43</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>14:41:47</t>
+          <t>15:02:50</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
@@ -1570,12 +1537,12 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>9.83</t>
+          <t>10.04</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>14:42:25</t>
+          <t>15:02:57</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1612,7 +1579,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Meta description found: 'A new Flutter project.'</t>
+          <t>Meta description found: 'DermaSense AI – AI-powered skin disease detection and dermatology assistance platform'</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1622,12 +1589,12 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>4.29</t>
+          <t>5.88</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>14:42:35</t>
+          <t>15:03:08</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
@@ -1674,12 +1641,12 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>6.22</t>
+          <t>6.35</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>14:42:40</t>
+          <t>15:03:14</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -1706,7 +1673,7 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Direct URL access to login route works</t>
+          <t>Direct URL access to all core routes works</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1716,7 +1683,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Direct URL access OK: https://dermasense-ai-18698.web.app/#/login</t>
+          <t>All core routes loaded successfully via direct URL access</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1726,17 +1693,17 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>16.04</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>14:42:46</t>
+          <t>15:03:20</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>https://dermasense-ai-18698.web.app/#/login</t>
+          <t>https://dermasense-ai-18698.web.app/#/dashboard</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
@@ -1768,105 +1735,105 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>DermaSense AI  -  Selenium Test Summary</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Tested URL</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>https://dermasense-ai-18698.web.app</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Total Test Cases</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>FAILED</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Pass Rate</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
-        <is>
-          <t>50.0%</t>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Run Date/Time</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>2026-06-11  14:42:52</t>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-14  15:03:39</t>
         </is>
       </c>
     </row>

</xml_diff>